<commit_message>
fix(frontend): แก้ไข import Stock
</commit_message>
<xml_diff>
--- a/fixdesk-frontend/public/example/TemplateExcelStock.xlsx
+++ b/fixdesk-frontend/public/example/TemplateExcelStock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pachara\Team0\fixdesk-system\fixdesk-frontend\public\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837B331D-9317-424E-B30D-9AF4665D8304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF04E11-7465-4766-9309-4B21F880211D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,31 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
-  <si>
-    <t>ชื่อผู้ใช้งาน</t>
-  </si>
-  <si>
-    <t>นามสกุลผู้ใช้งาน</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Lastname</t>
-  </si>
-  <si>
-    <t>000-000-0000</t>
-  </si>
-  <si>
-    <t>000-000-0001</t>
-  </si>
-  <si>
-    <t>000-000-0002</t>
-  </si>
-  <si>
-    <t>หน่วยงาน.........</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>หมายเหตุ: ช่องที่มีเครื่องหมาย * เป็นข้อมูลบังคับที่จำเป็นต้องระบุ</t>
   </si>
@@ -133,6 +109,21 @@
       </rPr>
       <t>*</t>
     </r>
+  </si>
+  <si>
+    <t>TV</t>
+  </si>
+  <si>
+    <t>Tv123</t>
+  </si>
+  <si>
+    <t>ไฟฟ้า</t>
+  </si>
+  <si>
+    <t>ชิ้น</t>
+  </si>
+  <si>
+    <t>พร้อมใช้งาน</t>
   </si>
 </sst>
 </file>
@@ -221,7 +212,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -553,25 +544,25 @@
   <sheetData>
     <row r="1" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K1" s="5"/>
       <c r="M1" s="7"/>
@@ -583,68 +574,44 @@
     </row>
     <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>3</v>
+      <c r="D2" s="2">
+        <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="N3" s="7"/>
     </row>
     <row r="4" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>

</xml_diff>